<commit_message>
Add Close/Confidence Check sheet to free lite P&L
Ship the updated lite workbook with a first Close sheet (monthly
checklist + Confidence Check) and a How-to step that starts there.
Landing copy and README mention the Close sheet. Polar, Pro, and the
quarterly workbook are unchanged.

Co-authored-by: Jreed1235TER <Jreed1235TER@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/solopreneur-pl-lite.xlsx
+++ b/solopreneur-pl-lite.xlsx
@@ -7,14 +7,15 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Setup" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Monthly" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Annual" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="How to use" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Close" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Setup" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Monthly" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Annual" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="How to use" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Monthly'!$A$5:$Q$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Monthly'!$1:$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Monthly'!$A$5:$Q$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Monthly'!$1:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +26,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,8 +81,19 @@
       <color rgb="001A1916"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -128,6 +140,16 @@
         <fgColor rgb="00DCE6DF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -169,7 +191,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -235,6 +257,14 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -598,6 +628,343 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="78" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>Monthly close — Confidence Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="29" t="inlineStr">
+        <is>
+          <t>Turn the calculator into a habit. Do this once per month before you trust profit or tax set-aside. Yellow = you type. Green-gray = formula.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Month to close (1=Jan … 12=Dec)</t>
+        </is>
+      </c>
+      <c r="B4" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Change this number; Confidence Check below follows Monthly row for that month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Last closed (date)</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="n"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Type the date you finished this close.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="31" t="inlineStr">
+        <is>
+          <t>MONTHLY CLOSE CHECKLIST</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>Done? (Yes/No)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1. Import / paste</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Bank/export or invoices pasted or typed into this month’s yellow revenue &amp; expense cells on Monthly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2. Categorize</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Every amount sits in a named category (not dumped only in Other). If unsure, park in Other and note below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>3. Owner draws</t>
+        </is>
+      </c>
+      <c r="B10" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Owner draws / personal transfers recorded (use Other expense or note $ in B16). Not the same as profit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>4. See profit</t>
+        </is>
+      </c>
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Read Profit before set-aside for this month (formula below).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>5. See tax set-aside</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Read Tax / set-aside $ for this month; move that cash to your tax parking account if that is your habit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="31" t="inlineStr">
+        <is>
+          <t>CONFIDENCE CHECK (trust the number?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Uncategorized / unknown expenses $</t>
+        </is>
+      </c>
+      <c r="B15" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Type any spend still not categorized. Ideal = 0 before you trust profit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Owner draws this month $</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Draws you took. Reminder only — does not change Monthly formulas unless you also booked them as expenses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Missing income? (Yes/No)</t>
+        </is>
+      </c>
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Any unpaid invoices or Stripe payouts not in revenue yet?</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="31" t="inlineStr">
+        <is>
+          <t>COMPUTED FROM MONTHLY (do not edit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Revenue (this month)</t>
+        </is>
+      </c>
+      <c r="B21" s="32">
+        <f>IF(B4&lt;1,"",IF(B4&gt;12,"",INDEX(Monthly!E6:E17,B4)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Expenses (this month)</t>
+        </is>
+      </c>
+      <c r="B22" s="32">
+        <f>IF(B4&lt;1,"",IF(B4&gt;12,"",INDEX(Monthly!M6:M17,B4)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Profit before set-aside</t>
+        </is>
+      </c>
+      <c r="B23" s="32">
+        <f>IF(B4&lt;1,"",IF(B4&gt;12,"",INDEX(Monthly!N6:N17,B4)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Tax / set-aside $</t>
+        </is>
+      </c>
+      <c r="B24" s="32">
+        <f>IF(B4&lt;1,"",IF(B4&gt;12,"",INDEX(Monthly!O6:O17,B4)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Profit after set-aside</t>
+        </is>
+      </c>
+      <c r="B25" s="32">
+        <f>IF(B4&lt;1,"",IF(B4&gt;12,"",INDEX(Monthly!P6:P17,B4)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Largest expense category $</t>
+        </is>
+      </c>
+      <c r="B26" s="32">
+        <f>IF(B4&lt;1,"",IF(B4&gt;12,"",MAX(INDEX(Monthly!F6:L17,B4,0))))</f>
+        <v/>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>If one category dominates, sanity-check it before you trust the month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Expense share of revenue</t>
+        </is>
+      </c>
+      <c r="B27" s="32">
+        <f>IF(B4&lt;1,"",IF(B4&gt;12,"",IF(B21="","",IF(B21=0,"n/a",ROUND(B22/B21,2)))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Confidence flags</t>
+        </is>
+      </c>
+      <c r="B28" s="33">
+        <f>IF(B4&lt;1,"",IF(B4&gt;12,"",IF(B15&gt;0,"Uncategorized $ still open. ","")&amp;IF(COUNTIF(B17,"Y*")&gt;0,"Missing income flagged. ","")&amp;IF(COUNTIF(B8:B12,"Yes")&lt;5,"Checklist incomplete. ","")&amp;IF(B15&gt;0,"Review flags before parking tax cash.",IF(COUNTIF(B17,"N*")&lt;1,"Review flags before parking tax cash.",IF(COUNTIF(B8:B12,"Yes")&lt;5,"Review flags before parking tax cash.","OK to trust this month’s profit/set-aside (still not tax advice).")))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="29" t="inlineStr">
+        <is>
+          <t>Habit loop: Close this sheet → fix flags → read set-aside → park cash → set Last closed date. Pair with the quarterly workbook when the quarter ends.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="29" t="inlineStr">
+        <is>
+          <t>Not tax, legal, or accounting advice. Built by an AI agent working for Jeremy Reed.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B28:F28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="001F3D32"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
@@ -623,8 +990,6 @@
           <t>EXAMPLE workbook — yellow cells are inputs. Replace them with your numbers. Green-gray cells are formulas. Do not type over formulas.</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -716,7 +1081,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
       <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Computed (formula)</t>
@@ -741,7 +1105,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="004A2C1A"/>
@@ -783,22 +1147,6 @@
           <t>Empty revenue or expense cells count as 0. Do not type in green-gray columns (those are SUM / IF / ROUND formulas). Tax rate and owner-pay target live on Setup.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
-      <c r="O2" s="2" t="n"/>
-      <c r="P2" s="2" t="n"/>
-      <c r="Q2" s="2" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="13" t="inlineStr"/>
@@ -807,29 +1155,16 @@
           <t>REVENUE — type amounts; blank = 0</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
       <c r="F4" s="15" t="inlineStr">
         <is>
           <t>EXPENSES — type amounts; blank = 0</t>
         </is>
       </c>
-      <c r="G4" s="15" t="n"/>
-      <c r="H4" s="15" t="n"/>
-      <c r="I4" s="15" t="n"/>
-      <c r="J4" s="15" t="n"/>
-      <c r="K4" s="15" t="n"/>
-      <c r="L4" s="15" t="n"/>
-      <c r="M4" s="15" t="n"/>
       <c r="N4" s="16" t="inlineStr">
         <is>
           <t>COMPUTED — formulas (do not edit)</t>
         </is>
       </c>
-      <c r="O4" s="16" t="n"/>
-      <c r="P4" s="16" t="n"/>
-      <c r="Q4" s="16" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
@@ -1751,7 +2086,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001A2A3A"/>
@@ -1778,7 +2113,6 @@
           <t>Pulled from Monthly YEAR TOTAL and Setup. EXAMPLE year until you replace the yellow cells.</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -1938,14 +2272,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="005C574E"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -1966,69 +2300,83 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="27" t="inlineStr">
-        <is>
-          <t>1. Open this file in Excel or Google Sheets (File → Import in Sheets). Macros are not used.</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>0. Each month open the Close sheet first: run the checklist + Confidence Check, then trust Monthly profit / set-aside.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>2. On Setup, set Business name, Year, and Tax / set-aside % (one cell, e.g. 0.30). Optional: owner pay target and starting cash.</t>
+          <t>1. Open this file in Excel or Google Sheets (File → Import in Sheets). Macros are not used.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>3. This is a set-aside planner, not a tax filing tool. The % is what you want to park, not a prepared return.</t>
+          <t>2. On Setup, set Business name, Year, and Tax / set-aside % (one cell, e.g. 0.30). Optional: owner pay target and starting cash.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>4. On Monthly, replace the EXAMPLE yellow cells with this year’s revenue and expenses. Leave a cell blank if it is zero.</t>
+          <t>3. This is a set-aside planner, not a tax filing tool. The % is what you want to park, not a prepared return.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>5. Read each month’s Tax / set-aside and Profit after set-aside. Those columns are formulas — do not type over them.</t>
+          <t>4. On Monthly, replace the EXAMPLE yellow cells with this year’s revenue and expenses. Leave a cell blank if it is zero.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>6. Annual pulls the year totals. Change Setup!B6 and every month’s set-aside updates.</t>
+          <t>5. Read each month’s Tax / set-aside and Profit after set-aside. Those columns are formulas — do not type over them.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="27" t="inlineStr">
         <is>
+          <t>6. Annual pulls the year totals. Change Setup!B6 and every month’s set-aside updates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
           <t>7. Built by an AI agent working for Jeremy Reed. Not tax, legal, or accounting advice.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Yellow = you type. Green-gray = formula (SUM / IF / ROUND only). No VBA, no macros, no spilled arrays.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Not tax, legal, or accounting advice. Built by an AI agent working for Jeremy Reed.</t>
         </is>
       </c>
     </row>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A4:B4"/>

</xml_diff>

<commit_message>
Add free Close/Confidence Check sheet to lite P&L
Ship the updated lite workbook with a first Close sheet (monthly
checklist + Confidence Check) and a How-to step that starts there.
Landing copy and README mention the Close sheet. Polar, Pro, and the
quarterly workbook are unchanged.

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: Jreed1235TER <Jreed1235TER@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/solopreneur-pl-lite.xlsx
+++ b/solopreneur-pl-lite.xlsx
@@ -7,14 +7,15 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Setup" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Monthly" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Annual" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="How to use" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Close" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Setup" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Monthly" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Annual" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="How to use" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Monthly'!$A$5:$Q$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Monthly'!$1:$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Monthly'!$A$5:$Q$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Monthly'!$1:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +26,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,8 +81,19 @@
       <color rgb="001A1916"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -128,6 +140,16 @@
         <fgColor rgb="00DCE6DF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -169,7 +191,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -235,6 +257,14 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -598,6 +628,343 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="78" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>Monthly close — Confidence Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="29" t="inlineStr">
+        <is>
+          <t>Turn the calculator into a habit. Do this once per month before you trust profit or tax set-aside. Yellow = you type. Green-gray = formula.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Month to close (1=Jan … 12=Dec)</t>
+        </is>
+      </c>
+      <c r="B4" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Change this number; Confidence Check below follows Monthly row for that month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Last closed (date)</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="n"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Type the date you finished this close.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="31" t="inlineStr">
+        <is>
+          <t>MONTHLY CLOSE CHECKLIST</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>Done? (Yes/No)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1. Import / paste</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Bank/export or invoices pasted or typed into this month’s yellow revenue &amp; expense cells on Monthly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2. Categorize</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Every amount sits in a named category (not dumped only in Other). If unsure, park in Other and note below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>3. Owner draws</t>
+        </is>
+      </c>
+      <c r="B10" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Owner draws / personal transfers recorded (use Other expense or note $ in B16). Not the same as profit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>4. See profit</t>
+        </is>
+      </c>
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Read Profit before set-aside for this month (formula below).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>5. See tax set-aside</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Read Tax / set-aside $ for this month; move that cash to your tax parking account if that is your habit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="31" t="inlineStr">
+        <is>
+          <t>CONFIDENCE CHECK (trust the number?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Uncategorized / unknown expenses $</t>
+        </is>
+      </c>
+      <c r="B15" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Type any spend still not categorized. Ideal = 0 before you trust profit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Owner draws this month $</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Draws you took. Reminder only — does not change Monthly formulas unless you also booked them as expenses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Missing income? (Yes/No)</t>
+        </is>
+      </c>
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Any unpaid invoices or Stripe payouts not in revenue yet?</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="31" t="inlineStr">
+        <is>
+          <t>COMPUTED FROM MONTHLY (do not edit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Revenue (this month)</t>
+        </is>
+      </c>
+      <c r="B21" s="32">
+        <f>IF(B4&lt;1,"",IF(B4&gt;12,"",INDEX(Monthly!E6:E17,B4)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Expenses (this month)</t>
+        </is>
+      </c>
+      <c r="B22" s="32">
+        <f>IF(B4&lt;1,"",IF(B4&gt;12,"",INDEX(Monthly!M6:M17,B4)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Profit before set-aside</t>
+        </is>
+      </c>
+      <c r="B23" s="32">
+        <f>IF(B4&lt;1,"",IF(B4&gt;12,"",INDEX(Monthly!N6:N17,B4)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Tax / set-aside $</t>
+        </is>
+      </c>
+      <c r="B24" s="32">
+        <f>IF(B4&lt;1,"",IF(B4&gt;12,"",INDEX(Monthly!O6:O17,B4)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Profit after set-aside</t>
+        </is>
+      </c>
+      <c r="B25" s="32">
+        <f>IF(B4&lt;1,"",IF(B4&gt;12,"",INDEX(Monthly!P6:P17,B4)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Largest expense category $</t>
+        </is>
+      </c>
+      <c r="B26" s="32">
+        <f>IF(B4&lt;1,"",IF(B4&gt;12,"",MAX(INDEX(Monthly!F6:L17,B4,0))))</f>
+        <v/>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>If one category dominates, sanity-check it before you trust the month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Expense share of revenue</t>
+        </is>
+      </c>
+      <c r="B27" s="32">
+        <f>IF(B4&lt;1,"",IF(B4&gt;12,"",IF(B21="","",IF(B21=0,"n/a",ROUND(B22/B21,2)))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Confidence flags</t>
+        </is>
+      </c>
+      <c r="B28" s="33">
+        <f>IF(B4&lt;1,"",IF(B4&gt;12,"",IF(B15&gt;0,"Uncategorized $ still open. ","")&amp;IF(COUNTIF(B17,"Y*")&gt;0,"Missing income flagged. ","")&amp;IF(COUNTIF(B8:B12,"Yes")&lt;5,"Checklist incomplete. ","")&amp;IF(B15&gt;0,"Review flags before parking tax cash.",IF(COUNTIF(B17,"N*")&lt;1,"Review flags before parking tax cash.",IF(COUNTIF(B8:B12,"Yes")&lt;5,"Review flags before parking tax cash.","OK to trust this month’s profit/set-aside (still not tax advice).")))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="29" t="inlineStr">
+        <is>
+          <t>Habit loop: Close this sheet → fix flags → read set-aside → park cash → set Last closed date. Pair with the quarterly workbook when the quarter ends.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="29" t="inlineStr">
+        <is>
+          <t>Not tax, legal, or accounting advice. Built by an AI agent working for Jeremy Reed.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B28:F28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="001F3D32"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
@@ -623,8 +990,6 @@
           <t>EXAMPLE workbook — yellow cells are inputs. Replace them with your numbers. Green-gray cells are formulas. Do not type over formulas.</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -716,7 +1081,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
       <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Computed (formula)</t>
@@ -741,7 +1105,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="004A2C1A"/>
@@ -783,22 +1147,6 @@
           <t>Empty revenue or expense cells count as 0. Do not type in green-gray columns (those are SUM / IF / ROUND formulas). Tax rate and owner-pay target live on Setup.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
-      <c r="O2" s="2" t="n"/>
-      <c r="P2" s="2" t="n"/>
-      <c r="Q2" s="2" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="13" t="inlineStr"/>
@@ -807,29 +1155,16 @@
           <t>REVENUE — type amounts; blank = 0</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
       <c r="F4" s="15" t="inlineStr">
         <is>
           <t>EXPENSES — type amounts; blank = 0</t>
         </is>
       </c>
-      <c r="G4" s="15" t="n"/>
-      <c r="H4" s="15" t="n"/>
-      <c r="I4" s="15" t="n"/>
-      <c r="J4" s="15" t="n"/>
-      <c r="K4" s="15" t="n"/>
-      <c r="L4" s="15" t="n"/>
-      <c r="M4" s="15" t="n"/>
       <c r="N4" s="16" t="inlineStr">
         <is>
           <t>COMPUTED — formulas (do not edit)</t>
         </is>
       </c>
-      <c r="O4" s="16" t="n"/>
-      <c r="P4" s="16" t="n"/>
-      <c r="Q4" s="16" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
@@ -1751,7 +2086,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001A2A3A"/>
@@ -1778,7 +2113,6 @@
           <t>Pulled from Monthly YEAR TOTAL and Setup. EXAMPLE year until you replace the yellow cells.</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -1938,14 +2272,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="005C574E"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -1966,69 +2300,83 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="27" t="inlineStr">
-        <is>
-          <t>1. Open this file in Excel or Google Sheets (File → Import in Sheets). Macros are not used.</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>0. Each month open the Close sheet first: run the checklist + Confidence Check, then trust Monthly profit / set-aside.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>2. On Setup, set Business name, Year, and Tax / set-aside % (one cell, e.g. 0.30). Optional: owner pay target and starting cash.</t>
+          <t>1. Open this file in Excel or Google Sheets (File → Import in Sheets). Macros are not used.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>3. This is a set-aside planner, not a tax filing tool. The % is what you want to park, not a prepared return.</t>
+          <t>2. On Setup, set Business name, Year, and Tax / set-aside % (one cell, e.g. 0.30). Optional: owner pay target and starting cash.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>4. On Monthly, replace the EXAMPLE yellow cells with this year’s revenue and expenses. Leave a cell blank if it is zero.</t>
+          <t>3. This is a set-aside planner, not a tax filing tool. The % is what you want to park, not a prepared return.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>5. Read each month’s Tax / set-aside and Profit after set-aside. Those columns are formulas — do not type over them.</t>
+          <t>4. On Monthly, replace the EXAMPLE yellow cells with this year’s revenue and expenses. Leave a cell blank if it is zero.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>6. Annual pulls the year totals. Change Setup!B6 and every month’s set-aside updates.</t>
+          <t>5. Read each month’s Tax / set-aside and Profit after set-aside. Those columns are formulas — do not type over them.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="27" t="inlineStr">
         <is>
+          <t>6. Annual pulls the year totals. Change Setup!B6 and every month’s set-aside updates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
           <t>7. Built by an AI agent working for Jeremy Reed. Not tax, legal, or accounting advice.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Yellow = you type. Green-gray = formula (SUM / IF / ROUND only). No VBA, no macros, no spilled arrays.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Not tax, legal, or accounting advice. Built by an AI agent working for Jeremy Reed.</t>
         </is>
       </c>
     </row>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A4:B4"/>

</xml_diff>